<commit_message>
docs(example): regenerate the exports with the quotation's terms on the invoice
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WqoocMczx3spPPqhrRpAE5
</commit_message>
<xml_diff>
--- a/docs/example/invoice-export.xlsx
+++ b/docs/example/invoice-export.xlsx
@@ -58,10 +58,10 @@
     <t>Q-00001/GNS/X/2026</t>
   </si>
   <si>
-    <t>2026-10-10</t>
-  </si>
-  <si>
-    <t>2026-11-09</t>
+    <t>2026-10-11</t>
+  </si>
+  <si>
+    <t>2026-11-10</t>
   </si>
   <si>
     <t>PT Samudra Contoh Nusantara</t>

</xml_diff>

<commit_message>
docs(example): regenerate the exports with the new PDF layout
The examples now show the halved margins, the smaller logo and number,
the shared summary rows (Total Rp18.510.000, Diskon Produk 5%
-Rp888.000, Sub Total Rp17.622.000) and the real invoice signer.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WqoocMczx3spPPqhrRpAE5
</commit_message>
<xml_diff>
--- a/docs/example/invoice-export.xlsx
+++ b/docs/example/invoice-export.xlsx
@@ -58,10 +58,10 @@
     <t>Q-00001/GNS/X/2026</t>
   </si>
   <si>
-    <t>2026-10-11</t>
-  </si>
-  <si>
-    <t>2026-11-10</t>
+    <t>2026-10-12</t>
+  </si>
+  <si>
+    <t>2026-11-11</t>
   </si>
   <si>
     <t>PT Samudra Contoh Nusantara</t>

</xml_diff>